<commit_message>
docs: regenerate the examples without the gain holes
Both causes are fixed, so every bar now has an unbroken gain profile.
The mpv span also gains two samples and a slightly different median, as
the collapsed beat it covers now counts for the three samples it stands
for rather than one.
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -621,7 +621,7 @@
         <v>0.53</v>
       </c>
       <c r="L2">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -653,13 +653,13 @@
         <v>0.315</v>
       </c>
       <c r="J3">
-        <v>0.338</v>
+        <v>0.3395</v>
       </c>
       <c r="K3">
         <v>0.35</v>
       </c>
       <c r="L3">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:13">

</xml_diff>

<commit_message>
feat: a second host in the fixture, and far more variety
The tree is host-partitioned so machines can share it, and the fixture
only ever had one -- so nothing exercised the thing phase 6 was mostly
about. It now carries ce2 and ce3, each with its own chain, verified
separately.

They have different habits, which is what makes a host filter worth
having: ce2 is evenings through the Scarlett, ce3 is a laptop with
daytime browser listening on headphones, shorter and quieter. They
overlap on sixteen occasions, so the report has genuine concurrent spans
-- two machines playing at once is two sources of sound.

Days now carry one to four sessions rather than one or two, spread
across the working day as well as the evening: 261 spans against 106,
three players, three output devices. Still a pure function of host and
date, so regenerating changes nothing.
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="72">
   <si>
     <t>Host</t>
   </si>
@@ -59,19 +59,64 @@
     <t>In quiet hours</t>
   </si>
   <si>
+    <t>ce3</t>
+  </si>
+  <si>
+    <t>2026-10-18T09:40:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-18T11:30:00+02:00</t>
+  </si>
+  <si>
+    <t>1h50m</t>
+  </si>
+  <si>
+    <t>firefox</t>
+  </si>
+  <si>
+    <t>Nils Frahm — Says (Live)</t>
+  </si>
+  <si>
+    <t>Nils Frahm</t>
+  </si>
+  <si>
+    <t>https://youtube.com/watch?v=dIww</t>
+  </si>
+  <si>
+    <t>alsa_output.pci-0000_00_1f.3.analog-stereo</t>
+  </si>
+  <si>
+    <t>2026-10-18T13:40:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-18T15:10:00+02:00</t>
+  </si>
+  <si>
+    <t>1h30m</t>
+  </si>
+  <si>
+    <t>mpd</t>
+  </si>
+  <si>
+    <t>Spiegel im Spiegel</t>
+  </si>
+  <si>
+    <t>Arvo Pärt</t>
+  </si>
+  <si>
+    <t>sync/part/spiegel.flac</t>
+  </si>
+  <si>
     <t>ce2</t>
   </si>
   <si>
-    <t>2026-10-18T18:00:00+02:00</t>
-  </si>
-  <si>
-    <t>2026-10-18T20:30:00+02:00</t>
-  </si>
-  <si>
-    <t>2h30m</t>
-  </si>
-  <si>
-    <t>mpd</t>
+    <t>2026-10-18T21:00:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-18T23:40:00+02:00</t>
+  </si>
+  <si>
+    <t>2h40m</t>
   </si>
   <si>
     <t>Harmony of Difference</t>
@@ -86,25 +131,7 @@
     <t>alsa_output.usb-Focusrite_Scarlett_4i4_USB-00.pro-output-0</t>
   </si>
   <si>
-    <t>2026-10-18T21:10:00+02:00</t>
-  </si>
-  <si>
-    <t>2026-10-18T22:40:00+02:00</t>
-  </si>
-  <si>
-    <t>1h30m</t>
-  </si>
-  <si>
-    <t>II (Continuous Mix)</t>
-  </si>
-  <si>
-    <t>Voices from the Lake</t>
-  </si>
-  <si>
-    <t>sync/vftl/11.flac</t>
-  </si>
-  <si>
-    <t>40m00s</t>
+    <t>1h40m</t>
   </si>
   <si>
     <t>2026-10-19T21:15:00+02:00</t>
@@ -113,9 +140,6 @@
     <t>2026-10-19T23:05:00+02:00</t>
   </si>
   <si>
-    <t>1h50m</t>
-  </si>
-  <si>
     <t>Discreet Music</t>
   </si>
   <si>
@@ -128,9 +152,48 @@
     <t>1h05m</t>
   </si>
   <si>
+    <t>2026-10-20T14:00:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-20T16:40:00+02:00</t>
+  </si>
+  <si>
+    <t>mpv</t>
+  </si>
+  <si>
+    <t>Stalker (1979)</t>
+  </si>
+  <si>
+    <t>Andrei Tarkovsky</t>
+  </si>
+  <si>
+    <t>/media/films/stalker.mkv</t>
+  </si>
+  <si>
+    <t>2026-10-20T20:30:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-20T21:50:00+02:00</t>
+  </si>
+  <si>
+    <t>1h20m</t>
+  </si>
+  <si>
+    <t>A Rainbow in Curved Air</t>
+  </si>
+  <si>
+    <t>Terry Riley</t>
+  </si>
+  <si>
+    <t>sync/riley/rainbow.flac</t>
+  </si>
+  <si>
     <t>Hosts</t>
   </si>
   <si>
+    <t>ce2, ce3</t>
+  </si>
+  <si>
     <t>Window</t>
   </si>
   <si>
@@ -146,7 +209,7 @@
     <t>Chain</t>
   </si>
   <si>
-    <t>intact (2932 lines)</t>
+    <t>intact (6099 lines)</t>
   </si>
   <si>
     <t>ce2 2026-10-18</t>
@@ -155,10 +218,19 @@
     <t>dfn not yet stamped, digicert not yet stamped</t>
   </si>
   <si>
+    <t>ce3 2026-10-18</t>
+  </si>
+  <si>
     <t>ce2 2026-10-19</t>
   </si>
   <si>
+    <t>ce2 2026-10-20</t>
+  </si>
+  <si>
     <t>ce2 2026-10-21</t>
+  </si>
+  <si>
+    <t>ce3 2026-10-21</t>
   </si>
 </sst>
 </file>
@@ -508,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -598,16 +670,16 @@
         <v>22</v>
       </c>
       <c r="J2">
-        <v>0.44</v>
+        <v>0.197</v>
       </c>
       <c r="K2">
-        <v>0.477</v>
+        <v>0.23399999999999999</v>
       </c>
       <c r="L2">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="M2">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -624,78 +696,201 @@
         <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I3" t="s">
         <v>22</v>
       </c>
       <c r="J3">
-        <v>0.47</v>
+        <v>0.25</v>
       </c>
       <c r="K3">
-        <v>0.4935</v>
+        <v>0.2595</v>
       </c>
       <c r="L3">
-        <v>0.52</v>
+        <v>0.27</v>
       </c>
       <c r="M3">
         <v>20</v>
       </c>
-      <c r="N3" s="2" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4">
+        <v>0.42</v>
+      </c>
+      <c r="K4">
+        <v>0.546</v>
+      </c>
+      <c r="L4">
+        <v>0.68</v>
+      </c>
+      <c r="M4">
+        <v>34</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5">
+        <v>0.34</v>
+      </c>
+      <c r="K5">
+        <v>0.3895</v>
+      </c>
+      <c r="L5">
+        <v>0.42</v>
+      </c>
+      <c r="M5">
+        <v>24</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6">
+        <v>0.315</v>
+      </c>
+      <c r="K6">
+        <v>0.34</v>
+      </c>
+      <c r="L6">
+        <v>0.35</v>
+      </c>
+      <c r="M6">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7">
+        <v>0.41</v>
+      </c>
+      <c r="K7">
+        <v>0.44</v>
+      </c>
+      <c r="L7">
+        <v>0.47</v>
+      </c>
+      <c r="M7">
         <v>18</v>
-      </c>
-      <c r="F4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4">
-        <v>0.34</v>
-      </c>
-      <c r="K4">
-        <v>0.3895</v>
-      </c>
-      <c r="L4">
-        <v>0.42</v>
-      </c>
-      <c r="M4">
-        <v>24</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -705,7 +900,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -714,58 +909,82 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: group the timeline by month, collapse the anchor footer
The gutter showed a full date plus hostname in 5rem, so it wrapped --
and the host span used a class scoped to table cells, so it rendered
inline and ran into the date: "2026-08-01ce2". Rows are now grouped
under a month heading and carry only day, weekday and host, with the
axis repeated per month so it stays near the rows it labels.

The anchor footer listed every day of every host: a hundred and
forty-five rows saying the same thing, which buries the one row that
does not. Consecutive days reporting the same status collapse into a
single line naming the span. A day whose token failed verification is
always listed alone and breaks the run around it, because that is the
line a reader has to see -- checked by planting a file that looks like
a token and is not.
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
   <si>
     <t>Host</t>
   </si>
@@ -182,16 +182,10 @@
     <t>intact (5069 lines)</t>
   </si>
   <si>
-    <t>ce2 2026-10-18</t>
+    <t>ce2 2026-10-18 … 2026-10-20  (3 days)</t>
   </si>
   <si>
     <t>dfn not yet stamped, digicert not yet stamped</t>
-  </si>
-  <si>
-    <t>ce2 2026-10-19</t>
-  </si>
-  <si>
-    <t>ce2 2026-10-20</t>
   </si>
   <si>
     <t>ce3 2026-10-21</t>
@@ -829,7 +823,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -884,22 +878,6 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" t="s">
-        <v>56</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: the example tree plays records track by track
The demo wrote one span per album, so the examples never contained the
case the timeline now has to draw: tracks following one another closely
enough that the page would collide them. The library carries real track
listings instead -- Reich's sections at two to seven minutes, Riley's two
sides at nineteen and twenty-two, Basinski's single hour-long piece -- and
a session lays a record across itself, starting wherever the needle landed
and pausing now and then for whoever got up to change it.

The beat had to go with it. A span ends at the last beat that saw the
track, so at a five-minute beat a four-minute song came back as a span of
no length at all. A session now beats every minute, which is nearer what
the daemon really does, and costs almost nothing: the gain is still read
on the five-minute grid, so the beats inside one step are identical and
collapse to the single rewritten line they would have been anyway.
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="111">
   <si>
     <t>Host</t>
   </si>
@@ -65,10 +65,10 @@
     <t>2026-10-18T14:40:00+02:00</t>
   </si>
   <si>
-    <t>2026-10-18T16:40:00+02:00</t>
-  </si>
-  <si>
-    <t>2h00m</t>
+    <t>2026-10-18T16:44:00+02:00</t>
+  </si>
+  <si>
+    <t>2h04m</t>
   </si>
   <si>
     <t>mpv</t>
@@ -89,82 +89,232 @@
     <t>2026-10-18T19:20:00+02:00</t>
   </si>
   <si>
-    <t>2026-10-18T20:25:00+02:00</t>
-  </si>
-  <si>
-    <t>1h05m</t>
+    <t>2026-10-18T19:50:00+02:00</t>
+  </si>
+  <si>
+    <t>30m00s</t>
   </si>
   <si>
     <t>mpd</t>
   </si>
   <si>
-    <t>The Disintegration Loops I</t>
+    <t>Discreet Music</t>
+  </si>
+  <si>
+    <t>Brian Eno</t>
+  </si>
+  <si>
+    <t>sync/eno/01.flac</t>
+  </si>
+  <si>
+    <t>2026-10-18T19:51:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-18T19:59:00+02:00</t>
+  </si>
+  <si>
+    <t>8m00s</t>
+  </si>
+  <si>
+    <t>Fullness of Wind</t>
+  </si>
+  <si>
+    <t>sync/eno/02.flac</t>
+  </si>
+  <si>
+    <t>2026-10-18T20:00:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-18T20:04:00+02:00</t>
+  </si>
+  <si>
+    <t>4m00s</t>
+  </si>
+  <si>
+    <t>French Catalogues</t>
+  </si>
+  <si>
+    <t>sync/eno/03.flac</t>
+  </si>
+  <si>
+    <t>2026-10-18T20:05:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-18T20:11:00+02:00</t>
+  </si>
+  <si>
+    <t>6m00s</t>
+  </si>
+  <si>
+    <t>Brutal Ardour</t>
+  </si>
+  <si>
+    <t>sync/eno/04.flac</t>
+  </si>
+  <si>
+    <t>2026-10-18T20:12:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-18T20:26:00+02:00</t>
+  </si>
+  <si>
+    <t>14m00s</t>
+  </si>
+  <si>
+    <t>2026-10-19T20:30:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T21:32:00+02:00</t>
+  </si>
+  <si>
+    <t>1h02m</t>
+  </si>
+  <si>
+    <t>dlp 1.1</t>
   </si>
   <si>
     <t>William Basinski</t>
   </si>
   <si>
-    <t>sync/basinski/dlp1.flac</t>
-  </si>
-  <si>
-    <t>2026-10-19T20:30:00+02:00</t>
-  </si>
-  <si>
-    <t>2026-10-19T21:40:00+02:00</t>
-  </si>
-  <si>
-    <t>1h10m</t>
-  </si>
-  <si>
-    <t>Discreet Music</t>
-  </si>
-  <si>
-    <t>Brian Eno</t>
-  </si>
-  <si>
-    <t>sync/eno/discreet.flac</t>
+    <t>sync/basinski/01.flac</t>
+  </si>
+  <si>
+    <t>2026-10-19T21:36:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T21:42:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T21:51:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T21:54:00+02:00</t>
+  </si>
+  <si>
+    <t>3m00s</t>
+  </si>
+  <si>
+    <t>Knowledge</t>
+  </si>
+  <si>
+    <t>Kamasi Washington</t>
+  </si>
+  <si>
+    <t>sync/kamasi/03.flac</t>
   </si>
   <si>
     <t>2026-10-19T21:55:00+02:00</t>
   </si>
   <si>
-    <t>2026-10-19T22:45:00+02:00</t>
-  </si>
-  <si>
-    <t>50m00s</t>
-  </si>
-  <si>
-    <t>A Rainbow in Curved Air</t>
-  </si>
-  <si>
-    <t>Terry Riley</t>
-  </si>
-  <si>
-    <t>sync/riley/rainbow.flac</t>
-  </si>
-  <si>
-    <t>45m00s</t>
+    <t>2026-10-19T21:58:00+02:00</t>
+  </si>
+  <si>
+    <t>Perspective</t>
+  </si>
+  <si>
+    <t>sync/kamasi/04.flac</t>
+  </si>
+  <si>
+    <t>2026-10-19T21:59:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:03:00+02:00</t>
+  </si>
+  <si>
+    <t>Integrity</t>
+  </si>
+  <si>
+    <t>sync/kamasi/05.flac</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:04:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:16:00+02:00</t>
+  </si>
+  <si>
+    <t>12m00s</t>
+  </si>
+  <si>
+    <t>Truth</t>
+  </si>
+  <si>
+    <t>sync/kamasi/06.flac</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:17:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:20:00+02:00</t>
+  </si>
+  <si>
+    <t>Desire</t>
+  </si>
+  <si>
+    <t>sync/kamasi/01.flac</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:24:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:27:00+02:00</t>
+  </si>
+  <si>
+    <t>Humility</t>
+  </si>
+  <si>
+    <t>sync/kamasi/02.flac</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:28:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:31:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:32:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:35:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:36:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:40:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:41:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:53:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:54:00+02:00</t>
+  </si>
+  <si>
+    <t>2026-10-19T22:56:00+02:00</t>
+  </si>
+  <si>
+    <t>2m00s</t>
   </si>
   <si>
     <t>2026-10-20T21:45:00+02:00</t>
   </si>
   <si>
-    <t>2026-10-20T23:50:00+02:00</t>
-  </si>
-  <si>
-    <t>2h05m</t>
-  </si>
-  <si>
-    <t>Symphony No. 3, Op. 36: II. Lento</t>
-  </si>
-  <si>
-    <t>Henryk Górecki</t>
-  </si>
-  <si>
-    <t>sync/gorecki/02.flac</t>
-  </si>
-  <si>
-    <t>1h50m</t>
+    <t>2026-10-20T23:49:00+02:00</t>
+  </si>
+  <si>
+    <t>II (Continuous Mix)</t>
+  </si>
+  <si>
+    <t>Voices from the Lake</t>
+  </si>
+  <si>
+    <t>sync/vftl/01.flac</t>
+  </si>
+  <si>
+    <t>1h49m</t>
   </si>
   <si>
     <t>Hosts</t>
@@ -188,7 +338,7 @@
     <t>Chain</t>
   </si>
   <si>
-    <t>intact (4720 lines)</t>
+    <t>intact (6853 lines)</t>
   </si>
   <si>
     <t>ce2 2026-10-18 … 2026-10-21  (4 days)</t>
@@ -547,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -640,13 +790,13 @@
         <v>0.317</v>
       </c>
       <c r="K2">
-        <v>0.34</v>
+        <v>0.341</v>
       </c>
       <c r="L2">
         <v>0.35</v>
       </c>
       <c r="M2">
-        <v>26</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -678,16 +828,16 @@
         <v>22</v>
       </c>
       <c r="J3">
-        <v>0.431</v>
+        <v>0.46</v>
       </c>
       <c r="K3">
-        <v>0.46</v>
+        <v>0.483</v>
       </c>
       <c r="L3">
         <v>0.489</v>
       </c>
       <c r="M3">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -710,25 +860,25 @@
         <v>33</v>
       </c>
       <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
         <v>34</v>
       </c>
-      <c r="H4" t="s">
-        <v>35</v>
-      </c>
       <c r="I4" t="s">
         <v>22</v>
       </c>
       <c r="J4">
-        <v>0.38</v>
+        <v>0.46</v>
       </c>
       <c r="K4">
-        <v>0.416</v>
+        <v>0.4665</v>
       </c>
       <c r="L4">
-        <v>0.44</v>
+        <v>0.473</v>
       </c>
       <c r="M4">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -736,43 +886,40 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
         <v>36</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>37</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>38</v>
       </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" t="s">
         <v>39</v>
       </c>
-      <c r="G5" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" t="s">
-        <v>41</v>
-      </c>
       <c r="I5" t="s">
         <v>22</v>
       </c>
       <c r="J5">
-        <v>0.4</v>
+        <v>0.447</v>
       </c>
       <c r="K5">
-        <v>0.44</v>
+        <v>0.447</v>
       </c>
       <c r="L5">
-        <v>0.46</v>
+        <v>0.447</v>
       </c>
       <c r="M5">
-        <v>11</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -780,43 +927,685 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
         <v>43</v>
       </c>
-      <c r="C6" t="s">
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="D6" t="s">
+      <c r="I6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6">
+        <v>0.431</v>
+      </c>
+      <c r="K6">
+        <v>0.437</v>
+      </c>
+      <c r="L6">
+        <v>0.437</v>
+      </c>
+      <c r="M6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
         <v>45</v>
       </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="C7" t="s">
         <v>46</v>
       </c>
-      <c r="G6" t="s">
+      <c r="D7" t="s">
         <v>47</v>
       </c>
-      <c r="H6" t="s">
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7">
+        <v>0.431</v>
+      </c>
+      <c r="K7">
+        <v>0.431</v>
+      </c>
+      <c r="L7">
+        <v>0.447</v>
+      </c>
+      <c r="M7">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
         <v>48</v>
       </c>
-      <c r="I6" t="s">
-        <v>22</v>
-      </c>
-      <c r="J6">
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8">
+        <v>0.385</v>
+      </c>
+      <c r="K8">
+        <v>0.422</v>
+      </c>
+      <c r="L8">
+        <v>0.44</v>
+      </c>
+      <c r="M8">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9">
+        <v>0.38</v>
+      </c>
+      <c r="K9">
+        <v>0.381</v>
+      </c>
+      <c r="L9">
+        <v>0.381</v>
+      </c>
+      <c r="M9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H10" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" t="s">
+        <v>22</v>
+      </c>
+      <c r="J10">
+        <v>0.43</v>
+      </c>
+      <c r="K10">
+        <v>0.43</v>
+      </c>
+      <c r="L10">
+        <v>0.43</v>
+      </c>
+      <c r="M10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11">
+        <v>0.439</v>
+      </c>
+      <c r="K11">
+        <v>0.439</v>
+      </c>
+      <c r="L11">
+        <v>0.439</v>
+      </c>
+      <c r="M11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" t="s">
+        <v>22</v>
+      </c>
+      <c r="J12">
+        <v>0.439</v>
+      </c>
+      <c r="K12">
+        <v>0.449</v>
+      </c>
+      <c r="L12">
+        <v>0.449</v>
+      </c>
+      <c r="M12">
+        <v>6</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" t="s">
+        <v>60</v>
+      </c>
+      <c r="H13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" t="s">
+        <v>22</v>
+      </c>
+      <c r="J13">
+        <v>0.449</v>
+      </c>
+      <c r="K13">
+        <v>0.4575</v>
+      </c>
+      <c r="L13">
+        <v>0.46</v>
+      </c>
+      <c r="M13">
+        <v>14</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J14">
+        <v>0.454</v>
+      </c>
+      <c r="K14">
+        <v>0.459</v>
+      </c>
+      <c r="L14">
+        <v>0.459</v>
+      </c>
+      <c r="M14">
+        <v>5</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>81</v>
+      </c>
+      <c r="G15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H15" t="s">
+        <v>82</v>
+      </c>
+      <c r="I15" t="s">
+        <v>22</v>
+      </c>
+      <c r="J15">
+        <v>0.446</v>
+      </c>
+      <c r="K15">
+        <v>0.446</v>
+      </c>
+      <c r="L15">
+        <v>0.454</v>
+      </c>
+      <c r="M15">
+        <v>5</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" t="s">
+        <v>60</v>
+      </c>
+      <c r="H16" t="s">
+        <v>61</v>
+      </c>
+      <c r="I16" t="s">
+        <v>22</v>
+      </c>
+      <c r="J16">
+        <v>0.436</v>
+      </c>
+      <c r="K16">
+        <v>0.446</v>
+      </c>
+      <c r="L16">
+        <v>0.446</v>
+      </c>
+      <c r="M16">
+        <v>5</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" t="s">
+        <v>60</v>
+      </c>
+      <c r="H17" t="s">
+        <v>65</v>
+      </c>
+      <c r="I17" t="s">
+        <v>22</v>
+      </c>
+      <c r="J17">
+        <v>0.424</v>
+      </c>
+      <c r="K17">
+        <v>0.436</v>
+      </c>
+      <c r="L17">
+        <v>0.436</v>
+      </c>
+      <c r="M17">
+        <v>5</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H18" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" t="s">
+        <v>22</v>
+      </c>
+      <c r="J18">
+        <v>0.414</v>
+      </c>
+      <c r="K18">
+        <v>0.424</v>
+      </c>
+      <c r="L18">
+        <v>0.424</v>
+      </c>
+      <c r="M18">
+        <v>6</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" t="s">
+        <v>73</v>
+      </c>
+      <c r="G19" t="s">
+        <v>60</v>
+      </c>
+      <c r="H19" t="s">
+        <v>74</v>
+      </c>
+      <c r="I19" t="s">
+        <v>22</v>
+      </c>
+      <c r="J19">
+        <v>0.401</v>
+      </c>
+      <c r="K19">
+        <v>0.406</v>
+      </c>
+      <c r="L19">
+        <v>0.414</v>
+      </c>
+      <c r="M19">
+        <v>14</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" t="s">
+        <v>60</v>
+      </c>
+      <c r="H20" t="s">
+        <v>78</v>
+      </c>
+      <c r="I20" t="s">
+        <v>22</v>
+      </c>
+      <c r="J20">
+        <v>0.4</v>
+      </c>
+      <c r="K20">
+        <v>0.4005</v>
+      </c>
+      <c r="L20">
+        <v>0.401</v>
+      </c>
+      <c r="M20">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" t="s">
+        <v>96</v>
+      </c>
+      <c r="G21" t="s">
+        <v>97</v>
+      </c>
+      <c r="H21" t="s">
+        <v>98</v>
+      </c>
+      <c r="I21" t="s">
+        <v>22</v>
+      </c>
+      <c r="J21">
         <v>0.42</v>
       </c>
-      <c r="K6">
+      <c r="K21">
         <v>0.554</v>
       </c>
-      <c r="L6">
-        <v>0.7</v>
-      </c>
-      <c r="M6">
-        <v>27</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>49</v>
+      <c r="L21">
+        <v>0.689</v>
+      </c>
+      <c r="M21">
+        <v>127</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -835,50 +1624,50 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B1" t="s">
-        <v>51</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
style: reports write dates day first
23-10-2026 is how a reader parses a date: between two rows of the same
month the day is the field that differs, and it should be the one the eye
lands on. The leading-year form is for sorting, and nothing in a report is
sorted by reading its text.

Where something is sorted by it, ISO stays -- the data- attributes the
filters group and compare by, the two exports, the JSON, and the integrity
table's day list, which is sorted as strings before it is collapsed into
runs and only reformatted on the way out.

The window label in the title is left alone too: it echoes the span as it
was asked for on the command line, and a title that no longer matches the
command that produced it trades one legibility for a worse loss.
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -341,13 +341,13 @@
     <t>intact (6853 lines)</t>
   </si>
   <si>
-    <t>ce2 2026-10-18 … 2026-10-21  (4 days)</t>
+    <t>ce2 18-10-2026 … 21-10-2026  (4 days)</t>
   </si>
   <si>
     <t>dfn not yet stamped, digicert not yet stamped</t>
   </si>
   <si>
-    <t>ce3 2026-10-18 … 2026-10-21  (4 days)</t>
+    <t>ce3 18-10-2026 … 21-10-2026  (4 days)</t>
   </si>
 </sst>
 </file>

</xml_diff>